<commit_message>
Stop GS OPS VIS NOW drawing over other sections (bug #8)
Add an onSectionLeave() hook that showSection() runs for the section
being left. GS OPS uses it to turn VIS NOW off, so its 10 s refresh
timer stops and it no longer redraws its status panel and key into
#default under other sections.

Also fix the gsOpsDefaultAvailable() guard, which matched the GS OPS
spine button instead of the section and so always passed. And stop
toggleVisibleSats() starting the timer if the user left while the
catalogue was loading.

Mark bug #8 fixed in bugsDB.xlsx.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bugsDB.xlsx
+++ b/bugsDB.xlsx
@@ -1307,12 +1307,12 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>GS OPS key keeps reappearing in the control panel after switching to ON-ORBIT</t>
+          <t>GS OPS key keeps reappearing on top of other control-panel displays after GS OPS has been visited</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -1322,30 +1322,34 @@
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>Control area — assets/gsOpsPanel.js (VIS NOW status panel) / assets/onOrbitPanel.js</t>
+          <t>Control area – assets/gsOpsPanel.js (VIS NOW status panel), affects all sections</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>After visiting the GS OPS section and then switching to ON-ORBIT, the GS OPS key (the link-state colour key from the VIS NOW status panel) keeps popping up in the control panel, in place of ON-ORBIT's own content (the orbit regime table).</t>
+          <t>Once the GS OPS section has been opened once via the LCARS spine, the GS OPS key (the link-state colour key from the VIS NOW status panel) keeps re-appearing in the control panel on top of other sections' displays (e.g. ON-ORBIT's orbit regime table). First seen with ON-ORBIT on 2026-10-10; broadened 2026-10-20: it happens with any other control-panel display.</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>1. Open GS OPS (VIS NOW on). 2. Click ON-ORBIT in the left menu. 3. Watch the control panel.</t>
+          <t>1. Open GS OPS from the LCARS spine (VIS NOW on). 2. Open any other section from the spine (e.g. ON-ORBIT). 3. Watch the control panel.</t>
         </is>
       </c>
       <c r="H9" s="8" t="inlineStr">
         <is>
-          <t>Once ON-ORBIT is open, its control panel shows only the orbit regime table; nothing from GS OPS appears.</t>
+          <t>After leaving GS OPS, the control panel shows only the current section's own content; nothing from GS OPS appears.</t>
         </is>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
-          <t>The GS OPS key repeatedly reappears in the control panel while ON-ORBIT is open.</t>
+          <t>The GS OPS key repeatedly reappears on top of the current section's control-panel display, in every section, for the rest of the visit.</t>
         </is>
       </c>
-      <c r="J9" s="8" t="n"/>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>UNCONFIRMED (code reading only, 2026-10-20; not yet checked in the browser). gsOpsDefaultAvailable() (gsOpsPanel.js:1184) uses document.querySelector('[data-section="gs-ops"]') without the 'main ' prefix, so it matches the GS OPS spine button (index.html:64), not the section div. showSection() only sets style.display on 'main [data-section]', so the button's style.display is '' and the guard always passes. The VIS NOW refresh timer (setInterval(renderVisibleSats, 10000), gsOpsPanel.js:1345) is only cleared when VIS NOW is toggled off, not when you leave GS OPS, so every 10 s it redraws the status panel and key into #default over whichever section is open. Needs VIS NOW switched on (it starts off). Suggested fix: use 'main [data-section="gs-ops"]'; optionally also skip or pause the timer's work while GS OPS is hidden.</t>
+        </is>
+      </c>
       <c r="K9" s="2" t="n">
         <v>46305</v>
       </c>
@@ -1359,7 +1363,9 @@
           <t>Al</t>
         </is>
       </c>
-      <c r="N9" s="2" t="n"/>
+      <c r="N9" s="2" t="n">
+        <v>46315</v>
+      </c>
       <c r="O9" s="5" t="inlineStr">
         <is>
           <t>Pre-Alpha</t>
@@ -1372,7 +1378,7 @@
       </c>
       <c r="Q9" s="8" t="inlineStr">
         <is>
-          <t>Root cause not yet investigated. Unconfirmed suspect: VIS NOW's 10-second refresh timer (gsOpsPanel.js) keeps running after leaving GS OPS and redraws its status panel into #default.</t>
+          <t>Fixed on DEV 2026-10-20; Al checked it in the browser. (1) lcars.js: onSectionLeave(sectionId, fn) registry; showSection() runs the leave hook of the visible section when switching to a different one. (2) gsOpsPanel.js registers a gs-ops hook that turns VIS NOW off (stops the timer, clears the map layer and status panel); VIS NOW reads OFF on return. (3) Guard selector fixed to 'main [data-section="gs-ops"]' as a backstop. (4) toggleVisibleSats() no longer starts the timer if the user left GS OPS while the catalogue was loading. Related, not fixed: GRD-TRACK live-position and terminator timers also keep running while hidden; they could use the same hook.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bug log: #9 SatNOGS frequencies on 9xxxx placeholder rows (fixed by DB refactor)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bugsDB.xlsx
+++ b/bugsDB.xlsx
@@ -1382,23 +1382,86 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="7" t="n"/>
-      <c r="B10" s="8" t="n"/>
-      <c r="C10" s="8" t="n"/>
-      <c r="D10" s="8" t="n"/>
-      <c r="E10" s="8" t="n"/>
-      <c r="F10" s="8" t="n"/>
-      <c r="G10" s="8" t="n"/>
-      <c r="H10" s="8" t="n"/>
-      <c r="I10" s="8" t="n"/>
-      <c r="J10" s="8" t="n"/>
-      <c r="K10" s="2" t="n"/>
-      <c r="L10" s="8" t="n"/>
-      <c r="M10" s="8" t="n"/>
-      <c r="N10" s="2" t="n"/>
-      <c r="O10" s="8" t="n"/>
-      <c r="Q10" s="8" t="n"/>
+    <row r="10" ht="135" customHeight="1" s="9">
+      <c r="A10" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>SatNOGS radio frequencies attached to SatNOGS's 9xxxx placeholder rows, not the real NORAD objects</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Ingestion – SatNOGS radio frequencies (scripts/ingestSatnogsRf.py, now scripts/publishSite.py); affects link budget and object details</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>SatNOGS radio frequencies (downlink/uplink, bandwidth, mode, baud) were attached to SatNOGS's duplicate rows under its own 98xxx/99xxx placeholder numbers instead of the real NORAD objects. Those NORAD objects therefore had no real frequencies, and the link budget fell back to band mid-points for them. On LIVE, 384 satellites' frequencies sat on 9xxxx duplicates (of 1,677 with SatNOGS frequencies).</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>1. On the pre-refactor data, query orbital_objects for rows with rfSource = 'satnogs' and noradID &gt;= 90000. 2. Look up the real NORAD object with the same international designator (e.g. SatNOGS 98193 JACK-007 = 2026-229K). 3. Compare their frequency columns.</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>Each satellite's SatNOGS frequencies are on its NORAD object, and SatNOGS's placeholder numbers never appear as separate objects.</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>Frequencies sat on the placeholder duplicate rows; the real NORAD objects had none.</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>The old pipeline (ingestOrbitalData.py) stored SatNOGS TLE rows as orbital objects under SatNOGS's placeholder numbers, and ingestSatnogsRf.py attached RF by the transmitter's norad_cat_id, which for satellites launched since NORAD's 5-digit numbers ran out (July 2026) is the placeholder, not the NORAD number.</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="L10" s="8" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="M10" s="8" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="O10" s="5" t="inlineStr">
+        <is>
+          <t>Pre-Alpha</t>
+        </is>
+      </c>
+      <c r="P10" s="5" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="Q10" s="8" t="inlineStr">
+        <is>
+          <t>Fixed by the database refactor (0_documentation/dbRefactorPlan.md, step 9): orbits come from Space-Track only, SatNOGS's TLE feed is kept only as an ID crosswalk, and publishSite.py links each transmitter by norad_follow_id, then the designator in SatNOGS's TLE matched to Space-Track's objectID, then its own norad_cat_id. After: 1,433 satellites with SatNOGS frequencies, none on 9xxxx duplicates. Live on LIVE since the migration, 2026-10-21 23:04 UTC. Covered by 0_tests/test_publishSite.py.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n"/>

</xml_diff>

<commit_message>
Bug 10 (.htaccess gap after DB refactor) fixed on LIVE: bug log, design doc security, plan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bugsDB.xlsx
+++ b/bugsDB.xlsx
@@ -1463,23 +1463,86 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="7" t="n"/>
-      <c r="B11" s="8" t="n"/>
-      <c r="C11" s="8" t="n"/>
-      <c r="D11" s="8" t="n"/>
-      <c r="E11" s="8" t="n"/>
-      <c r="F11" s="8" t="n"/>
-      <c r="G11" s="8" t="n"/>
-      <c r="H11" s="8" t="n"/>
-      <c r="I11" s="8" t="n"/>
-      <c r="J11" s="8" t="n"/>
-      <c r="K11" s="2" t="n"/>
-      <c r="L11" s="8" t="n"/>
-      <c r="M11" s="8" t="n"/>
-      <c r="N11" s="2" t="n"/>
-      <c r="O11" s="8" t="n"/>
-      <c r="Q11" s="8" t="n"/>
+    <row r="11" ht="135" customHeight="1" s="9">
+      <c r="A11" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Site .db.prev files and databases/.writers.lock downloadable after DB refactor (bug 7 regression)</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Live web server – .htaccess (server-only rewrite rules); databases/</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>After the database refactor moved the databases to databases/ and added .prev copies and a lock file, the live web server served some of them: databases/siteOrbital.db.prev and siteNews.db.prev (site databases, including Space-Track-derived data) and databases/.writers.lock returned 200. databases/siteOrbital.db itself was refused (403). A regression of bug 7.</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>1. curl -I https://gaps2024.com/LCARS-FAS/databases/siteOrbital.db.prev 2. Same for databases/siteNews.db.prev and databases/.writers.lock.</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>403 for every file under databases/ and every dot-file.</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>200 for the .db.prev files and .writers.lock (403 only for *.db).</t>
+        </is>
+      </c>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>The server-only .htaccess block list named the old folder ingestionDBs/ and the .db extension, but not databases/, the .prev/.tmp/.lock extensions or dot-files. The refactor added all of these without updating it.</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="n">
+        <v>46317</v>
+      </c>
+      <c r="L11" s="8" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="M11" s="8" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="n">
+        <v>46317</v>
+      </c>
+      <c r="O11" s="5" t="inlineStr">
+        <is>
+          <t>Pre-Alpha</t>
+        </is>
+      </c>
+      <c r="P11" s="5" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="Q11" s="8" t="inlineStr">
+        <is>
+          <t>Found by the DB refactor step 14 (documentation) session with HEAD requests. Fixed on LIVE 2026-10-22 ~11:55 UTC with Al's go-ahead: the folder rule adds databases/, the extension rule adds prev|tmp|new|lock|objects, and the dot-file rule is now (^|/)\. (covers .writers.lock, .referenceUpload/, .deployStage/). Backup: ~/backups/LCARS-FAS.htaccess.pre-dbRefactor-20261022-115511. Verified: siteOrbital.db, .db.prev, .db.tmp, .writers.lock and ingestionDBs/ return 403; pages and APIs 200. Regression guard: 0_tools/liveCheck.py privacy section, 15 private paths (commit 3800497). The .htaccess is a block list: any new file type or folder under the app root must be added to it and to liveCheck's privacy list.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n"/>

</xml_diff>

<commit_message>
EO panel: AREA imagery, filters, errors; space weather and DB refactor work
EO: TGT LOCN form gets an AREA selector (5-100 km); TGT FOCUS outlines the area and
downloads Sentinel-2 (Element 84) covering it from overviews, shown in its own map pane
so the country shapes no longer hide it. MAX CLOUD COVER and MAX LOOKBACK filters,
RESOLUTION as "this fine or better", SATELLITE moved, MATCHES label in the title bar,
red mid-map errors (NOT YET AVAILABLE, NO CLEAR SCENE, IMAGE FETCH FAILED), visualisation
class per source from Uhura's workbook (buildEoOptions.py), eoSelectorsTest.js.

Also commits earlier uncommitted work: space weather ingesters, charts and tests, the DB
refactor follow-ups, test harness updates, toDo.md.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bugsDB.xlsx
+++ b/bugsDB.xlsx
@@ -1544,23 +1544,84 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="7" t="n"/>
-      <c r="B12" s="8" t="n"/>
-      <c r="C12" s="8" t="n"/>
-      <c r="D12" s="8" t="n"/>
-      <c r="E12" s="8" t="n"/>
-      <c r="F12" s="8" t="n"/>
-      <c r="G12" s="8" t="n"/>
-      <c r="H12" s="8" t="n"/>
-      <c r="I12" s="8" t="n"/>
-      <c r="J12" s="8" t="n"/>
-      <c r="K12" s="2" t="n"/>
-      <c r="L12" s="8" t="n"/>
-      <c r="M12" s="8" t="n"/>
+    <row r="12" ht="135" customHeight="1" s="9">
+      <c r="A12" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Control panel scrolled off the top of the screen after clicking a spine button</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Spine navigation: assets/lcars.js showSection(); seen on EO</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>After clicking a spine button the new section loads, but the page is scrolled so that the control panel at the top is off the top of the screen. Intermittent: it does not happen every time. Definitely reproduced on the EO screen.</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>1. Open a section and scroll down the page, or use a tall section. 2. Click another button on the spine, for example EO. 3. Look at the top of the page.</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>Each spine click shows the new section with the control panel (and banner) visible at the top of the page.</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>The section's main content loads but the page stays scrolled down, leaving the control panel above the visible area.</t>
+        </is>
+      </c>
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>UNCONFIRMED: showSection() does not reset the scroll position. topFunction() (which scrolls to the top) is called from only two places in lcars.js, so most spine buttons keep whatever scroll position the previous section left. Map sections (EO) may also scroll the page when the map initialises. Not yet investigated.</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="L12" s="8" t="inlineStr">
+        <is>
+          <t>DEV</t>
+        </is>
+      </c>
+      <c r="M12" s="8" t="inlineStr">
+        <is>
+          <t>Al</t>
+        </is>
+      </c>
       <c r="N12" s="2" t="n"/>
-      <c r="O12" s="8" t="n"/>
-      <c r="Q12" s="8" t="n"/>
+      <c r="O12" s="5" t="inlineStr">
+        <is>
+          <t>Pre-Alpha</t>
+        </is>
+      </c>
+      <c r="P12" s="5" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="Q12" s="8" t="inlineStr">
+        <is>
+          <t>Fix applied 2026-10-24: showSection() now scrolls to the top on every section change. Awaiting Al's test on DEV; not yet marked Fixed. If it still happens on EO, suspect the map initialising and scrolling the page after showSection() has run.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n"/>

</xml_diff>